<commit_message>
docs: finalizar documentacion y entregar entregables del proyecto
- Se completa el PDF principal con las secciones desde Mantenimiento de software hasta Economia de Ingenieria de software.

- Se agrega el Excel Analisis_Costo_Beneficio_MenteSana_Web.xls, cronograma, EDT y diagrama de dominio.

- Proyecto terminado y listo para revision. ¡Muchas gracias, docente!
</commit_message>
<xml_diff>
--- a/Artefactos de Scrum Mente Sana.xlsx
+++ b/Artefactos de Scrum Mente Sana.xlsx
@@ -1,15 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\didie\Downloads\Necesario para software\Lo que hare\Proyecto Software\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE8E7B4-698D-4097-AC5E-C24116FDADCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Product Backlog" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Sprint Backlog" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Daily Scrum" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Retrospectiva" sheetId="4" r:id="rId8"/>
+    <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
+    <sheet name="Sprint Backlog" sheetId="2" r:id="rId2"/>
+    <sheet name="Daily Scrum" sheetId="3" r:id="rId3"/>
+    <sheet name="Retrospectiva" sheetId="4" r:id="rId4"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -489,55 +503,64 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="11">
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FF1F1F1F"/>
       <name val="&quot;Google Sans Text&quot;"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FF1F1F1F"/>
       <name val="&quot;Google Sans Text&quot;"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="&quot;Google Sans Text&quot;"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="&quot;Google Sans Text&quot;"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Google Sans"/>
     </font>
-    <font/>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Google Sans Text"/>
     </font>
@@ -547,7 +570,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -599,7 +622,13 @@
     </fill>
   </fills>
   <borders count="5">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -613,27 +642,34 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
+      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -643,121 +679,107 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="31">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="6" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="top"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="6" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="2" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="1" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="2" fillId="8" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="1" fillId="8" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="1" fillId="9" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -765,7 +787,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -955,28 +977,28 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Z1000"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="9.14"/>
-    <col customWidth="1" min="2" max="2" width="34.57"/>
-    <col customWidth="1" min="3" max="3" width="49.14"/>
-    <col customWidth="1" min="4" max="4" width="9.14"/>
-    <col customWidth="1" min="5" max="5" width="18.71"/>
-    <col customWidth="1" min="6" max="6" width="12.43"/>
-    <col customWidth="1" min="7" max="7" width="49.0"/>
-    <col customWidth="1" min="8" max="8" width="40.57"/>
-    <col customWidth="1" min="9" max="26" width="9.14"/>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="2" max="2" width="34.5703125" customWidth="1"/>
+    <col min="3" max="3" width="49.140625" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="49" customWidth="1"/>
+    <col min="8" max="8" width="40.5703125" customWidth="1"/>
+    <col min="9" max="26" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25.5" customHeight="1">
+    <row r="1" spans="1:26" ht="25.5" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1002,7 +1024,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="84.0" customHeight="1">
+    <row r="2" spans="1:26" ht="84" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -1016,7 +1038,7 @@
         <v>11</v>
       </c>
       <c r="E2" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>12</v>
@@ -1028,7 +1050,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" ht="83.25" customHeight="1">
+    <row r="3" spans="1:26" ht="83.25" customHeight="1">
       <c r="A3" s="3" t="s">
         <v>15</v>
       </c>
@@ -1042,7 +1064,7 @@
         <v>11</v>
       </c>
       <c r="E3" s="7">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>12</v>
@@ -1054,7 +1076,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" ht="118.5" customHeight="1">
+    <row r="4" spans="1:26" ht="118.5" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>20</v>
       </c>
@@ -1068,7 +1090,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="7">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>12</v>
@@ -1080,7 +1102,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" ht="76.5" customHeight="1">
+    <row r="5" spans="1:26" ht="76.5" customHeight="1">
       <c r="A5" s="3" t="s">
         <v>24</v>
       </c>
@@ -1094,7 +1116,7 @@
         <v>11</v>
       </c>
       <c r="E5" s="7">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>12</v>
@@ -1106,7 +1128,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" ht="123.75" customHeight="1">
+    <row r="6" spans="1:26" ht="123.75" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>28</v>
       </c>
@@ -1120,7 +1142,7 @@
         <v>11</v>
       </c>
       <c r="E6" s="7">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>12</v>
@@ -1132,7 +1154,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" ht="126.75" customHeight="1">
+    <row r="7" spans="1:26" ht="126.75" customHeight="1">
       <c r="A7" s="3" t="s">
         <v>32</v>
       </c>
@@ -1146,7 +1168,7 @@
         <v>35</v>
       </c>
       <c r="E7" s="7">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>12</v>
@@ -1158,7 +1180,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" ht="99.75" customHeight="1">
+    <row r="8" spans="1:26" ht="99.75" customHeight="1">
       <c r="A8" s="3" t="s">
         <v>37</v>
       </c>
@@ -1172,7 +1194,7 @@
         <v>11</v>
       </c>
       <c r="E8" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>12</v>
@@ -1189,7 +1211,7 @@
       <c r="L8" s="10"/>
       <c r="M8" s="10"/>
     </row>
-    <row r="9" ht="120.0" customHeight="1">
+    <row r="9" spans="1:26" ht="120" customHeight="1">
       <c r="A9" s="3" t="s">
         <v>42</v>
       </c>
@@ -1203,7 +1225,7 @@
         <v>35</v>
       </c>
       <c r="E9" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>12</v>
@@ -1233,7 +1255,7 @@
       <c r="Y9" s="10"/>
       <c r="Z9" s="10"/>
     </row>
-    <row r="10" ht="128.25" customHeight="1">
+    <row r="10" spans="1:26" ht="128.25" customHeight="1">
       <c r="A10" s="3" t="s">
         <v>46</v>
       </c>
@@ -1247,7 +1269,7 @@
         <v>11</v>
       </c>
       <c r="E10" s="7">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>12</v>
@@ -1277,7 +1299,7 @@
       <c r="Y10" s="10"/>
       <c r="Z10" s="10"/>
     </row>
-    <row r="11" ht="133.5" customHeight="1">
+    <row r="11" spans="1:26" ht="133.5" customHeight="1">
       <c r="A11" s="3" t="s">
         <v>50</v>
       </c>
@@ -1291,7 +1313,7 @@
         <v>11</v>
       </c>
       <c r="E11" s="7">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>12</v>
@@ -1321,7 +1343,7 @@
       <c r="Y11" s="10"/>
       <c r="Z11" s="10"/>
     </row>
-    <row r="12" ht="105.75" customHeight="1">
+    <row r="12" spans="1:26" ht="105.75" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>54</v>
       </c>
@@ -1335,7 +1357,7 @@
         <v>35</v>
       </c>
       <c r="E12" s="7">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>12</v>
@@ -1365,7 +1387,7 @@
       <c r="Y12" s="10"/>
       <c r="Z12" s="10"/>
     </row>
-    <row r="13" ht="95.25" customHeight="1">
+    <row r="13" spans="1:26" ht="95.25" customHeight="1">
       <c r="A13" s="3" t="s">
         <v>58</v>
       </c>
@@ -1379,7 +1401,7 @@
         <v>11</v>
       </c>
       <c r="E13" s="7">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>12</v>
@@ -1409,7 +1431,7 @@
       <c r="Y13" s="10"/>
       <c r="Z13" s="10"/>
     </row>
-    <row r="14" ht="120.75" customHeight="1">
+    <row r="14" spans="1:26" ht="120.75" customHeight="1">
       <c r="A14" s="11" t="s">
         <v>62</v>
       </c>
@@ -1423,7 +1445,7 @@
         <v>11</v>
       </c>
       <c r="E14" s="13">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="F14" s="13" t="s">
         <v>12</v>
@@ -1453,7 +1475,7 @@
       <c r="Y14" s="10"/>
       <c r="Z14" s="10"/>
     </row>
-    <row r="15">
+    <row r="15" spans="1:26" ht="114">
       <c r="A15" s="11" t="s">
         <v>66</v>
       </c>
@@ -1467,7 +1489,7 @@
         <v>11</v>
       </c>
       <c r="E15" s="13">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="F15" s="13" t="s">
         <v>12</v>
@@ -1497,7 +1519,7 @@
       <c r="Y15" s="10"/>
       <c r="Z15" s="10"/>
     </row>
-    <row r="16" ht="117.0" customHeight="1">
+    <row r="16" spans="1:26" ht="117" customHeight="1">
       <c r="A16" s="11" t="s">
         <v>70</v>
       </c>
@@ -1511,7 +1533,7 @@
         <v>11</v>
       </c>
       <c r="E16" s="13">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="F16" s="13" t="s">
         <v>12</v>
@@ -1541,7 +1563,7 @@
       <c r="Y16" s="10"/>
       <c r="Z16" s="10"/>
     </row>
-    <row r="17" ht="117.0" customHeight="1">
+    <row r="17" spans="1:8" ht="117" customHeight="1">
       <c r="A17" s="11" t="s">
         <v>75</v>
       </c>
@@ -1555,7 +1577,7 @@
         <v>11</v>
       </c>
       <c r="E17" s="13">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="F17" s="13" t="s">
         <v>12</v>
@@ -1567,18 +1589,18 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1"/>
-    <row r="22" ht="15.75" customHeight="1"/>
-    <row r="23" ht="15.75" customHeight="1"/>
-    <row r="24" ht="15.75" customHeight="1"/>
-    <row r="25" ht="15.75" customHeight="1"/>
-    <row r="26" ht="15.75" customHeight="1"/>
-    <row r="27" ht="15.75" customHeight="1"/>
-    <row r="28" ht="15.75" customHeight="1"/>
-    <row r="29" ht="15.75" customHeight="1"/>
-    <row r="30" ht="15.75" customHeight="1"/>
-    <row r="31" ht="15.75" customHeight="1"/>
-    <row r="32" ht="15.75" customHeight="1"/>
+    <row r="21" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="22" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="23" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="24" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="25" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="26" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="27" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="28" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="29" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="30" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="31" spans="1:8" ht="15.75" customHeight="1"/>
+    <row r="32" spans="1:8" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
@@ -2548,29 +2570,25 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:Z1000"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="21.0"/>
-    <col customWidth="1" min="2" max="2" width="36.71"/>
-    <col customWidth="1" min="3" max="3" width="13.57"/>
-    <col customWidth="1" min="4" max="4" width="17.14"/>
-    <col customWidth="1" min="5" max="5" width="17.86"/>
-    <col customWidth="1" min="6" max="24" width="9.14"/>
+    <col min="1" max="1" width="21" customWidth="1"/>
+    <col min="2" max="2" width="36.7109375" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.140625" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" customWidth="1"/>
+    <col min="6" max="24" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.0" customHeight="1">
+    <row r="1" spans="1:26" ht="33" customHeight="1">
       <c r="A1" s="14" t="s">
         <v>79</v>
       </c>
@@ -2587,7 +2605,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:26" ht="57">
       <c r="A2" s="11" t="s">
         <v>83</v>
       </c>
@@ -2598,7 +2616,7 @@
         <v>85</v>
       </c>
       <c r="D2" s="13">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="E2" s="13" t="s">
         <v>12</v>
@@ -2625,7 +2643,7 @@
       <c r="Y2" s="10"/>
       <c r="Z2" s="10"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:26" ht="28.5">
       <c r="A3" s="11" t="s">
         <v>8</v>
       </c>
@@ -2636,7 +2654,7 @@
         <v>87</v>
       </c>
       <c r="D3" s="13">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="E3" s="13" t="s">
         <v>12</v>
@@ -2663,7 +2681,7 @@
       <c r="Y3" s="10"/>
       <c r="Z3" s="10"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:26" ht="42.75">
       <c r="A4" s="11" t="s">
         <v>8</v>
       </c>
@@ -2674,7 +2692,7 @@
         <v>89</v>
       </c>
       <c r="D4" s="13">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="E4" s="13" t="s">
         <v>12</v>
@@ -2701,7 +2719,7 @@
       <c r="Y4" s="10"/>
       <c r="Z4" s="10"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:26" ht="57">
       <c r="A5" s="11" t="s">
         <v>62</v>
       </c>
@@ -2712,7 +2730,7 @@
         <v>89</v>
       </c>
       <c r="D5" s="13">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>12</v>
@@ -2739,7 +2757,7 @@
       <c r="Y5" s="10"/>
       <c r="Z5" s="10"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:26" ht="57">
       <c r="A6" s="11" t="s">
         <v>62</v>
       </c>
@@ -2750,7 +2768,7 @@
         <v>87</v>
       </c>
       <c r="D6" s="13">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>12</v>
@@ -2777,7 +2795,7 @@
       <c r="Y6" s="10"/>
       <c r="Z6" s="10"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:26" ht="42.75">
       <c r="A7" s="11" t="s">
         <v>37</v>
       </c>
@@ -2788,7 +2806,7 @@
         <v>87</v>
       </c>
       <c r="D7" s="13">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="E7" s="13" t="s">
         <v>12</v>
@@ -2815,7 +2833,7 @@
       <c r="Y7" s="10"/>
       <c r="Z7" s="10"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:26" ht="57">
       <c r="A8" s="11" t="s">
         <v>37</v>
       </c>
@@ -2826,7 +2844,7 @@
         <v>89</v>
       </c>
       <c r="D8" s="13">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="E8" s="13" t="s">
         <v>12</v>
@@ -2853,7 +2871,7 @@
       <c r="Y8" s="10"/>
       <c r="Z8" s="10"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:26" ht="57">
       <c r="A9" s="11" t="s">
         <v>37</v>
       </c>
@@ -2864,7 +2882,7 @@
         <v>85</v>
       </c>
       <c r="D9" s="13">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="E9" s="13" t="s">
         <v>12</v>
@@ -2891,7 +2909,7 @@
       <c r="Y9" s="10"/>
       <c r="Z9" s="10"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:26" ht="57">
       <c r="A10" s="11" t="s">
         <v>95</v>
       </c>
@@ -2902,7 +2920,7 @@
         <v>97</v>
       </c>
       <c r="D10" s="13">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="E10" s="13" t="s">
         <v>12</v>
@@ -2929,7 +2947,7 @@
       <c r="Y10" s="10"/>
       <c r="Z10" s="10"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:26" ht="71.25">
       <c r="A11" s="11" t="s">
         <v>83</v>
       </c>
@@ -2940,7 +2958,7 @@
         <v>87</v>
       </c>
       <c r="D11" s="13">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="E11" s="13" t="s">
         <v>12</v>
@@ -2967,68 +2985,68 @@
       <c r="Y11" s="10"/>
       <c r="Z11" s="10"/>
     </row>
-    <row r="21" ht="15.75" customHeight="1"/>
-    <row r="22" ht="15.75" customHeight="1">
+    <row r="21" spans="1:4" ht="15.75" customHeight="1"/>
+    <row r="22" spans="1:4" ht="15.75" customHeight="1">
       <c r="A22" s="16"/>
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
+    <row r="23" spans="1:4" ht="15.75" customHeight="1">
       <c r="A23" s="16"/>
       <c r="B23" s="16"/>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
+    <row r="24" spans="1:4" ht="15.75" customHeight="1">
       <c r="A24" s="16"/>
       <c r="B24" s="16"/>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
+    <row r="25" spans="1:4" ht="15.75" customHeight="1">
       <c r="A25" s="16"/>
       <c r="B25" s="16"/>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
+    <row r="26" spans="1:4" ht="15.75" customHeight="1">
       <c r="A26" s="16"/>
       <c r="B26" s="16"/>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
     </row>
-    <row r="27" ht="15.75" customHeight="1">
+    <row r="27" spans="1:4" ht="15.75" customHeight="1">
       <c r="A27" s="16"/>
       <c r="B27" s="16"/>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
+    <row r="28" spans="1:4" ht="15.75" customHeight="1">
       <c r="A28" s="16"/>
       <c r="B28" s="16"/>
       <c r="C28" s="16"/>
       <c r="D28" s="16"/>
     </row>
-    <row r="29" ht="15.75" customHeight="1">
+    <row r="29" spans="1:4" ht="15.75" customHeight="1">
       <c r="A29" s="16"/>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
       <c r="D29" s="16"/>
     </row>
-    <row r="30" ht="15.75" customHeight="1">
+    <row r="30" spans="1:4" ht="15.75" customHeight="1">
       <c r="A30" s="16"/>
       <c r="B30" s="16"/>
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
+    <row r="31" spans="1:4" ht="15.75" customHeight="1">
       <c r="A31" s="16"/>
       <c r="B31" s="16"/>
       <c r="C31" s="16"/>
       <c r="D31" s="16"/>
     </row>
-    <row r="32" ht="15.75" customHeight="1">
+    <row r="32" spans="1:4" ht="15.75" customHeight="1">
       <c r="A32" s="16"/>
       <c r="B32" s="16"/>
       <c r="C32" s="16"/>
@@ -4003,46 +4021,42 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:Z1000"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="16.71"/>
-    <col customWidth="1" min="2" max="2" width="49.57"/>
-    <col customWidth="1" min="3" max="3" width="22.71"/>
-    <col customWidth="1" min="4" max="4" width="28.43"/>
-    <col customWidth="1" min="5" max="24" width="9.14"/>
+    <col min="1" max="1" width="16.7109375" customWidth="1"/>
+    <col min="2" max="2" width="49.5703125" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" customWidth="1"/>
+    <col min="4" max="4" width="28.42578125" customWidth="1"/>
+    <col min="5" max="24" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:26">
+      <c r="A1" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="19"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="28"/>
     </row>
-    <row r="2">
-      <c r="A2" s="20" t="s">
+    <row r="2" spans="1:26">
+      <c r="A2" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="C2" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="17" t="s">
         <v>103</v>
       </c>
       <c r="E2" s="10"/>
@@ -4068,7 +4082,7 @@
       <c r="Y2" s="10"/>
       <c r="Z2" s="10"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:26" ht="71.25">
       <c r="A3" s="11" t="s">
         <v>85</v>
       </c>
@@ -4104,7 +4118,7 @@
       <c r="Y3" s="10"/>
       <c r="Z3" s="10"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:26" ht="85.5">
       <c r="A4" s="11" t="s">
         <v>89</v>
       </c>
@@ -4140,7 +4154,7 @@
       <c r="Y4" s="10"/>
       <c r="Z4" s="10"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:26" ht="71.25">
       <c r="A5" s="11" t="s">
         <v>87</v>
       </c>
@@ -4154,30 +4168,30 @@
         <v>111</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="21" t="s">
+    <row r="8" spans="1:26">
+      <c r="A8" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="19"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="28"/>
     </row>
-    <row r="9">
-      <c r="A9" s="22" t="s">
+    <row r="9" spans="1:26">
+      <c r="A9" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="E9" s="23"/>
+      <c r="E9" s="19"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:26" ht="71.25">
       <c r="A10" s="11" t="s">
         <v>85</v>
       </c>
@@ -4190,9 +4204,9 @@
       <c r="D10" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="E10" s="23"/>
+      <c r="E10" s="19"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:26" ht="85.5">
       <c r="A11" s="11" t="s">
         <v>89</v>
       </c>
@@ -4205,9 +4219,9 @@
       <c r="D11" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="E11" s="23"/>
+      <c r="E11" s="19"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:26" ht="85.5">
       <c r="A12" s="11" t="s">
         <v>87</v>
       </c>
@@ -4220,31 +4234,31 @@
       <c r="D12" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="E12" s="23"/>
+      <c r="E12" s="19"/>
     </row>
-    <row r="15">
-      <c r="A15" s="24" t="s">
+    <row r="15" spans="1:26">
+      <c r="A15" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="19"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="28"/>
     </row>
-    <row r="16">
-      <c r="A16" s="25" t="s">
+    <row r="16" spans="1:26">
+      <c r="A16" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="C16" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="D16" s="20" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:4" ht="85.5">
       <c r="A17" s="11" t="s">
         <v>85</v>
       </c>
@@ -4258,7 +4272,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:4" ht="85.5">
       <c r="A18" s="11" t="s">
         <v>89</v>
       </c>
@@ -4272,7 +4286,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:4" ht="99.75">
       <c r="A19" s="11" t="s">
         <v>87</v>
       </c>
@@ -4286,18 +4300,18 @@
         <v>128</v>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1"/>
-    <row r="22" ht="15.75" customHeight="1"/>
-    <row r="23" ht="15.75" customHeight="1"/>
-    <row r="24" ht="15.75" customHeight="1"/>
-    <row r="25" ht="15.75" customHeight="1"/>
-    <row r="26" ht="15.75" customHeight="1"/>
-    <row r="27" ht="15.75" customHeight="1"/>
-    <row r="28" ht="15.75" customHeight="1"/>
-    <row r="29" ht="15.75" customHeight="1"/>
-    <row r="30" ht="15.75" customHeight="1"/>
-    <row r="31" ht="15.75" customHeight="1"/>
-    <row r="32" ht="15.75" customHeight="1"/>
+    <row r="21" spans="1:4" ht="15.75" customHeight="1"/>
+    <row r="22" spans="1:4" ht="15.75" customHeight="1"/>
+    <row r="23" spans="1:4" ht="15.75" customHeight="1"/>
+    <row r="24" spans="1:4" ht="15.75" customHeight="1"/>
+    <row r="25" spans="1:4" ht="15.75" customHeight="1"/>
+    <row r="26" spans="1:4" ht="15.75" customHeight="1"/>
+    <row r="27" spans="1:4" ht="15.75" customHeight="1"/>
+    <row r="28" spans="1:4" ht="15.75" customHeight="1"/>
+    <row r="29" spans="1:4" ht="15.75" customHeight="1"/>
+    <row r="30" spans="1:4" ht="15.75" customHeight="1"/>
+    <row r="31" spans="1:4" ht="15.75" customHeight="1"/>
+    <row r="32" spans="1:4" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
@@ -5272,59 +5286,55 @@
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A15:D15"/>
   </mergeCells>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:Z1000"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="32.43"/>
-    <col customWidth="1" min="2" max="2" width="26.0"/>
-    <col customWidth="1" min="3" max="3" width="32.14"/>
-    <col customWidth="1" min="4" max="23" width="9.14"/>
+    <col min="1" max="1" width="32.42578125" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="3" max="3" width="32.140625" customWidth="1"/>
+    <col min="4" max="23" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30.75" customHeight="1">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:26" ht="30.75" customHeight="1">
+      <c r="A1" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="21" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="27" t="s">
+    <row r="2" spans="1:26" ht="71.25">
+      <c r="A2" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="28"/>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
-      <c r="N2" s="28"/>
-      <c r="O2" s="28"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
       <c r="P2" s="10"/>
       <c r="Q2" s="10"/>
       <c r="R2" s="10"/>
@@ -5337,28 +5347,28 @@
       <c r="Y2" s="10"/>
       <c r="Z2" s="10"/>
     </row>
-    <row r="3">
-      <c r="A3" s="27" t="s">
+    <row r="3" spans="1:26" ht="71.25">
+      <c r="A3" s="22" t="s">
         <v>135</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="22" t="s">
         <v>136</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-      <c r="I3" s="28"/>
-      <c r="J3" s="28"/>
-      <c r="K3" s="28"/>
-      <c r="L3" s="28"/>
-      <c r="M3" s="28"/>
-      <c r="N3" s="28"/>
-      <c r="O3" s="28"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
       <c r="P3" s="10"/>
       <c r="Q3" s="10"/>
       <c r="R3" s="10"/>
@@ -5371,28 +5381,28 @@
       <c r="Y3" s="10"/>
       <c r="Z3" s="10"/>
     </row>
-    <row r="4">
-      <c r="A4" s="27" t="s">
+    <row r="4" spans="1:26" ht="71.25">
+      <c r="A4" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="28"/>
-      <c r="K4" s="28"/>
-      <c r="L4" s="28"/>
-      <c r="M4" s="28"/>
-      <c r="N4" s="28"/>
-      <c r="O4" s="28"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
       <c r="R4" s="10"/>
@@ -5405,28 +5415,28 @@
       <c r="Y4" s="10"/>
       <c r="Z4" s="10"/>
     </row>
-    <row r="5">
-      <c r="A5" s="27" t="s">
+    <row r="5" spans="1:26" ht="71.25">
+      <c r="A5" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="22" t="s">
         <v>143</v>
       </c>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="28"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="23"/>
+      <c r="L5" s="23"/>
+      <c r="M5" s="23"/>
+      <c r="N5" s="23"/>
+      <c r="O5" s="23"/>
       <c r="P5" s="10"/>
       <c r="Q5" s="10"/>
       <c r="R5" s="10"/>
@@ -5439,35 +5449,35 @@
       <c r="Y5" s="10"/>
       <c r="Z5" s="10"/>
     </row>
-    <row r="6">
-      <c r="A6" s="27" t="s">
+    <row r="6" spans="1:26" ht="85.5">
+      <c r="A6" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="C6" s="27" t="s">
+      <c r="C6" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="29"/>
-      <c r="K6" s="29"/>
-      <c r="L6" s="29"/>
-      <c r="M6" s="29"/>
-      <c r="N6" s="29"/>
-      <c r="O6" s="29"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="24"/>
+      <c r="M6" s="24"/>
+      <c r="N6" s="24"/>
+      <c r="O6" s="24"/>
     </row>
-    <row r="7">
-      <c r="A7" s="30"/>
-      <c r="B7" s="30"/>
-      <c r="C7" s="30"/>
+    <row r="7" spans="1:26">
+      <c r="A7" s="25"/>
+      <c r="B7" s="25"/>
+      <c r="C7" s="25"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:26">
       <c r="G14" s="10"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -6451,9 +6461,7 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>